<commit_message>
Citas: Sofía confirma sola los trámites simples con cupo; agenda para repartirlas
- Cupo de citas por hora y feriados configurables en la hoja; los trámites
  marcados con «Revisión antes de la cita» siguen pendientes del personal.
- Si la hora está llena, Sofía ofrece las horas libres de ese día.
- Panel: pestaña Agenda por día para asignar cada cita a una persona,
  confirmar, cancelar o marcarla atendida.
- Resumen de las citas del día al WhatsApp del personal a las 07:00.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cms/Notaria41-contenido.xlsx
+++ b/cms/Notaria41-contenido.xlsx
@@ -652,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -666,7 +666,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -727,6 +727,11 @@
       </c>
       <c r="L1" s="4" t="inlineStr">
         <is>
+          <t>Revisión antes de la cita</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
           <t>Mostrar</t>
         </is>
       </c>
@@ -785,6 +790,11 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
@@ -839,6 +849,11 @@
       <c r="K3" s="5" t="inlineStr"/>
       <c r="L3" s="5" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
@@ -896,6 +911,11 @@
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
@@ -952,6 +972,11 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
@@ -1008,6 +1033,11 @@
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1077,6 +1107,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1128,6 +1163,11 @@
       </c>
       <c r="K8" s="5" t="inlineStr"/>
       <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1191,6 +1231,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1245,6 +1290,11 @@
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1310,6 +1360,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1365,6 +1420,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1420,6 +1480,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1478,6 +1543,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1532,6 +1602,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1581,6 +1656,11 @@
       <c r="J16" s="5" t="inlineStr"/>
       <c r="K16" s="5" t="inlineStr"/>
       <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1645,6 +1725,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1695,6 +1780,11 @@
       <c r="J18" s="5" t="inlineStr"/>
       <c r="K18" s="5" t="inlineStr"/>
       <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1758,6 +1848,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1815,6 +1910,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1867,6 +1967,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1920,6 +2025,11 @@
         </is>
       </c>
       <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -1985,6 +2095,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -2039,6 +2154,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -2097,6 +2217,11 @@
         </is>
       </c>
       <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -2162,6 +2287,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -2215,6 +2345,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -2267,6 +2402,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -2324,6 +2464,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -2377,6 +2522,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M30" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -2435,6 +2585,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -2488,6 +2643,11 @@
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M32" s="5" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
@@ -2541,6 +2701,11 @@
       <c r="K33" s="5" t="inlineStr"/>
       <c r="L33" s="5" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
@@ -2600,6 +2765,11 @@
         </is>
       </c>
       <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M34" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -2664,6 +2834,11 @@
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
@@ -2723,6 +2898,11 @@
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
@@ -2776,6 +2956,11 @@
       <c r="J37" s="5" t="inlineStr"/>
       <c r="K37" s="5" t="inlineStr"/>
       <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -2837,6 +3022,11 @@
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
@@ -2893,6 +3083,11 @@
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
@@ -2948,6 +3143,11 @@
         </is>
       </c>
       <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M40" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -3013,6 +3213,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -3071,6 +3276,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -3125,6 +3335,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -3178,6 +3393,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M44" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -3233,6 +3453,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M45" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -3290,6 +3515,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -3347,6 +3577,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -3398,6 +3633,11 @@
         </is>
       </c>
       <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="M48" s="5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -3458,9 +3698,14 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="G2:G248" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Porcentaje del SBU,Valor fijo (USD),Según cuantía,Consultar"</formula1>
     </dataValidation>
@@ -3472,6 +3717,9 @@
     </dataValidation>
     <dataValidation sqref="B2:B248" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"poderes,inmuebles,familia,herencias,declaraciones,empresas,diligencias"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:L500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3884,7 +4132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4130,6 +4378,26 @@
           <t>2026</t>
         </is>
       </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Citas por hora</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Feriados</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Portada: el nombre del notario como título, cargo encima y nuevo lema
- El h1 de la portada es «Dr. Dobri Miguel Albornoz Donoso», con el cargo
  («Notario Cuadragésimo Primero del Cantón Quito») encima y el lema
  «Fe pública al servicio de la comunidad.» debajo; se quita la frase de WhatsApp.
- La marca del menú muestra «Dr. Dobri Albornoz Donoso» y, en pequeño,
  «Notaría 41 · Quito» (se oculta en celulares angostos).
- Título de la página y og:title con el nombre del notario.
- notaria.json: cargo, notarioCorto y nuevo eslogan; la hoja acepta
  «Cargo del notario» en Configuración.
- Pruebas: Vitest para el cargo desde la hoja y Playwright para la portada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cms/Notaria41-contenido.xlsx
+++ b/cms/Notaria41-contenido.xlsx
@@ -4132,7 +4132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4178,167 +4178,171 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Eslogan</t>
+          <t>Cargo del notario</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Fe pública, con claridad.</t>
+          <t>Notario Cuadragésimo Primero del Cantón Quito</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Dirección</t>
+          <t>Eslogan</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Simón Bolívar Oe1-222, entre Juan Montalvo y Eugenio Espejo, frente al Parque Central de Tumbaco, Quito, Ecuador</t>
+          <t>Fe pública al servicio de la comunidad.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Teléfonos</t>
+          <t>Dirección</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>02 600 1141, 02 600 4141</t>
+          <t>Simón Bolívar Oe1-222, entre Juan Montalvo y Eugenio Espejo, frente al Parque Central de Tumbaco, Quito, Ecuador</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Teléfonos</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>593996530276</t>
+          <t>02 600 1141, 02 600 4141</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Correo</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>notaria41uio@gmail.com</t>
+          <t>593996530276</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Horario</t>
+          <t>Correo</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Lunes a viernes, de 08:00 a 17:00</t>
+          <t>notaria41uio@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Abre</t>
+          <t>Horario</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>Lunes a viernes, de 08:00 a 17:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Cierra</t>
+          <t>Abre</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>08:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Días de atención</t>
+          <t>Cierra</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>1,2,3,4,5</t>
+          <t>17:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Latitud</t>
+          <t>Días de atención</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>-0.2114</t>
+          <t>1,2,3,4,5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Longitud</t>
+          <t>Latitud</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>-78.4026</t>
+          <t>-0.2114</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Enlace para agendar</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr"/>
+          <t>Longitud</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>-78.4026</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/p/Notaria-41-Quito-100047615838049/</t>
-        </is>
-      </c>
+          <t>Enlace para agendar</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr"/>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/p/Notaria-41-Quito-100047615838049/</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr"/>
@@ -4346,58 +4350,66 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>SBU</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>482</t>
-        </is>
-      </c>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>IVA (%)</t>
+          <t>SBU</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>482</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Año de tarifas</t>
+          <t>IVA (%)</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Citas por hora</t>
+          <t>Año de tarifas</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2026</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
+          <t>Citas por hora</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
           <t>Feriados</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr"/>
+      <c r="B24" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Hoja: nombre corto del notario para el menú
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cms/Notaria41-contenido.xlsx
+++ b/cms/Notaria41-contenido.xlsx
@@ -4132,7 +4132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4190,167 +4190,171 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Eslogan</t>
+          <t>Nombre corto del notario</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Fe pública al servicio de la comunidad.</t>
+          <t>Dr. Dobri Albornoz Donoso</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Dirección</t>
+          <t>Eslogan</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Simón Bolívar Oe1-222, entre Juan Montalvo y Eugenio Espejo, frente al Parque Central de Tumbaco, Quito, Ecuador</t>
+          <t>Fe pública al servicio de la comunidad.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Teléfonos</t>
+          <t>Dirección</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>02 600 1141, 02 600 4141</t>
+          <t>Simón Bolívar Oe1-222, entre Juan Montalvo y Eugenio Espejo, frente al Parque Central de Tumbaco, Quito, Ecuador</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Teléfonos</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>593996530276</t>
+          <t>02 600 1141, 02 600 4141</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Correo</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>notaria41uio@gmail.com</t>
+          <t>593996530276</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Horario</t>
+          <t>Correo</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Lunes a viernes, de 08:00 a 17:00</t>
+          <t>notaria41uio@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Abre</t>
+          <t>Horario</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>Lunes a viernes, de 08:00 a 17:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Cierra</t>
+          <t>Abre</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>08:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Días de atención</t>
+          <t>Cierra</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>1,2,3,4,5</t>
+          <t>17:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Latitud</t>
+          <t>Días de atención</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>-0.2114</t>
+          <t>1,2,3,4,5</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Longitud</t>
+          <t>Latitud</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>-78.4026</t>
+          <t>-0.2114</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Enlace para agendar</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr"/>
+          <t>Longitud</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>-78.4026</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Facebook</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/p/Notaria-41-Quito-100047615838049/</t>
-        </is>
-      </c>
+          <t>Enlace para agendar</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr"/>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/p/Notaria-41-Quito-100047615838049/</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr"/>
@@ -4358,58 +4362,66 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>SBU</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>482</t>
-        </is>
-      </c>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>IVA (%)</t>
+          <t>SBU</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>482</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Año de tarifas</t>
+          <t>IVA (%)</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>15</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Citas por hora</t>
+          <t>Año de tarifas</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2026</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
+          <t>Citas por hora</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
           <t>Feriados</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr"/>
+      <c r="B25" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>